<commit_message>
Fixed issues in test data and accounting rule filters
</commit_message>
<xml_diff>
--- a/flsserver/src/FLS.Server.Tests/TestData/FlightInvoiceTestdata_SGN.xlsx
+++ b/flsserver/src/FLS.Server.Tests/TestData/FlightInvoiceTestdata_SGN.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="146">
   <si>
     <t>UseCase</t>
   </si>
@@ -325,9 +325,6 @@
   </si>
   <si>
     <t>Spring Hermann</t>
-  </si>
-  <si>
-    <t>2339-M</t>
   </si>
   <si>
     <t xml:space="preserve">Start und Landung Doppelsitzer Club-Segelflugzeug auf Homebase mit einem zweiten Piloten oder Passagier / Schlepp mit Club-eigenem Schleppflugzeug EXW und Turbo gebrauch </t>
@@ -480,6 +477,15 @@
   </si>
   <si>
     <t>1622-S</t>
+  </si>
+  <si>
+    <t>1593</t>
+  </si>
+  <si>
+    <t>EXW-FS-U</t>
+  </si>
+  <si>
+    <t>6203</t>
   </si>
 </sst>
 </file>
@@ -1393,7 +1399,7 @@
         <v>19</v>
       </c>
       <c r="U1" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="V1" s="2" t="s">
         <v>20</v>
@@ -1545,7 +1551,7 @@
         <v>80</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="J2" s="1">
         <v>1</v>
@@ -1605,7 +1611,7 @@
         <v>83</v>
       </c>
       <c r="AG2" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AH2" s="1">
         <v>0</v>
@@ -1658,7 +1664,7 @@
         <v>87</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="J3" s="1">
         <v>1</v>
@@ -1718,7 +1724,7 @@
         <v>83</v>
       </c>
       <c r="AG3" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AH3" s="1">
         <v>0</v>
@@ -1771,7 +1777,7 @@
         <v>74</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="J4" s="1">
         <v>1</v>
@@ -1780,7 +1786,7 @@
         <v>92</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="M4" s="1" t="s">
         <v>93</v>
@@ -1831,16 +1837,16 @@
         <v>92</v>
       </c>
       <c r="AF4" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AG4" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="AH4" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI4" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="AJ4" s="1">
         <v>20</v>
@@ -1887,7 +1893,7 @@
         <v>70</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="J5" s="1">
         <v>1</v>
@@ -1941,7 +1947,7 @@
         <v>1</v>
       </c>
       <c r="AD5" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AE5" s="1" t="s">
         <v>97</v>
@@ -1950,7 +1956,7 @@
         <v>99</v>
       </c>
       <c r="AG5" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="AH5" s="1">
         <v>0</v>
@@ -1965,30 +1971,21 @@
         <v>67</v>
       </c>
       <c r="AL5" s="5" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="AM5" s="1">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="AN5" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="AO5" s="5" t="s">
-        <v>86</v>
+      <c r="AO5" s="5">
+        <v>6203</v>
       </c>
       <c r="AP5" s="1">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AQ5" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AR5" s="5">
-        <v>6203</v>
-      </c>
-      <c r="AS5" s="1">
-        <v>1</v>
-      </c>
-      <c r="AT5" s="1" t="s">
         <v>68</v>
       </c>
     </row>
@@ -2000,7 +1997,7 @@
         <v>1</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>63</v>
@@ -2009,19 +2006,19 @@
         <v>81</v>
       </c>
       <c r="F6" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="J6" s="1">
+        <v>1</v>
+      </c>
+      <c r="K6" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="G6" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="J6" s="1">
-        <v>1</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>103</v>
-      </c>
       <c r="L6" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="O6" s="1" t="s">
         <v>98</v>
@@ -2042,10 +2039,10 @@
         <v>180</v>
       </c>
       <c r="U6">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="V6" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="W6" s="1" t="s">
         <v>85</v>
@@ -2069,13 +2066,13 @@
         <v>4</v>
       </c>
       <c r="AE6" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="AF6" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="AG6" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AH6" s="1">
         <v>0</v>
@@ -2090,10 +2087,10 @@
         <v>67</v>
       </c>
       <c r="AL6" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="AM6" s="1">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AN6" s="1" t="s">
         <v>67</v>
@@ -2125,31 +2122,31 @@
         <v>1</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>63</v>
       </c>
       <c r="E7" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>109</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>110</v>
       </c>
       <c r="J7" s="1">
         <v>3</v>
       </c>
       <c r="K7" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="M7" s="1" t="s">
         <v>111</v>
-      </c>
-      <c r="L7" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="M7" s="1" t="s">
-        <v>112</v>
       </c>
       <c r="P7" s="1">
         <v>60</v>
@@ -2170,7 +2167,7 @@
         <v>900</v>
       </c>
       <c r="V7" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="AC7" s="1">
         <v>1</v>
@@ -2179,13 +2176,13 @@
         <v>3</v>
       </c>
       <c r="AE7" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AF7" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="AG7" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AH7" s="1">
         <v>0</v>
@@ -2200,7 +2197,7 @@
         <v>67</v>
       </c>
       <c r="AL7" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="AM7" s="1">
         <v>15</v>
@@ -2226,7 +2223,7 @@
         <v>1</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>63</v>
@@ -2235,19 +2232,19 @@
         <v>88</v>
       </c>
       <c r="F8" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="J8" s="1">
+        <v>1</v>
+      </c>
+      <c r="K8" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="G8" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="J8" s="1">
-        <v>1</v>
-      </c>
-      <c r="K8" s="1" t="s">
-        <v>116</v>
-      </c>
       <c r="L8" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="P8" s="1">
         <v>61</v>
@@ -2265,7 +2262,7 @@
         <v>180</v>
       </c>
       <c r="U8">
-        <v>10</v>
+        <v>600</v>
       </c>
       <c r="V8" s="1" t="s">
         <v>72</v>
@@ -2292,13 +2289,13 @@
         <v>4</v>
       </c>
       <c r="AE8" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="AF8" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="AG8" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="AH8" s="1">
         <v>0</v>
@@ -2313,19 +2310,19 @@
         <v>67</v>
       </c>
       <c r="AL8" s="5" t="s">
-        <v>91</v>
+        <v>116</v>
       </c>
       <c r="AM8" s="1">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="AN8" s="1" t="s">
         <v>67</v>
       </c>
       <c r="AO8" s="5" t="s">
-        <v>117</v>
+        <v>91</v>
       </c>
       <c r="AP8" s="1">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="AQ8" s="1" t="s">
         <v>67</v>
@@ -2348,7 +2345,7 @@
         <v>1</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>63</v>
@@ -2357,19 +2354,19 @@
         <v>81</v>
       </c>
       <c r="F9" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="J9" s="1">
+        <v>1</v>
+      </c>
+      <c r="K9" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="G9" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="J9" s="1">
-        <v>1</v>
-      </c>
-      <c r="K9" s="1" t="s">
+      <c r="L9" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="L9" s="1" t="s">
-        <v>123</v>
       </c>
       <c r="P9" s="1">
         <v>60</v>
@@ -2390,7 +2387,7 @@
         <v>0</v>
       </c>
       <c r="V9" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="W9" s="1" t="s">
         <v>85</v>
@@ -2414,13 +2411,13 @@
         <v>2</v>
       </c>
       <c r="AE9" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="AF9" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="AF9" s="1" t="s">
-        <v>123</v>
-      </c>
       <c r="AG9" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AH9" s="1">
         <v>0</v>
@@ -2452,19 +2449,19 @@
         <v>1</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>63</v>
       </c>
       <c r="E10" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="G10" s="1" t="s">
         <v>128</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>129</v>
       </c>
       <c r="H10" s="3" t="s">
         <v>64</v>
@@ -2473,10 +2470,10 @@
         <v>1</v>
       </c>
       <c r="K10" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="L10" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="L10" s="1" t="s">
-        <v>123</v>
       </c>
       <c r="P10" s="1">
         <v>60</v>
@@ -2497,7 +2494,7 @@
         <v>0</v>
       </c>
       <c r="V10" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="W10" s="1" t="s">
         <v>77</v>
@@ -2521,19 +2518,19 @@
         <v>2</v>
       </c>
       <c r="AE10" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="AF10" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="AF10" s="1" t="s">
-        <v>123</v>
-      </c>
       <c r="AG10" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AH10" s="1">
         <v>0</v>
       </c>
-      <c r="AI10" s="5">
-        <v>3144</v>
+      <c r="AI10" s="5" t="s">
+        <v>143</v>
       </c>
       <c r="AJ10" s="1">
         <v>100</v>
@@ -2541,8 +2538,8 @@
       <c r="AK10" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="AL10" s="5">
-        <v>6200</v>
+      <c r="AL10" s="5" t="s">
+        <v>145</v>
       </c>
       <c r="AM10" s="1">
         <v>1</v>
@@ -2559,7 +2556,7 @@
         <v>1</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>63</v>
@@ -2568,19 +2565,19 @@
         <v>81</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="J11" s="1">
         <v>1</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="O11" s="1" t="s">
         <v>98</v>
@@ -2595,16 +2592,16 @@
         <v>84</v>
       </c>
       <c r="S11" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="T11" s="1">
         <v>180</v>
       </c>
       <c r="U11">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="V11" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="W11" s="1" t="s">
         <v>85</v>
@@ -2628,13 +2625,13 @@
         <v>3</v>
       </c>
       <c r="AE11" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="AF11" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="AG11" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AH11" s="1">
         <v>0</v>
@@ -2649,19 +2646,19 @@
         <v>67</v>
       </c>
       <c r="AL11" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="AM11" s="1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AN11" s="1" t="s">
         <v>67</v>
       </c>
       <c r="AO11" s="5" t="s">
-        <v>86</v>
+        <v>144</v>
       </c>
       <c r="AP11" s="1">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="AQ11" s="1" t="s">
         <v>67</v>
@@ -2672,7 +2669,7 @@
         <v>44</v>
       </c>
       <c r="B12" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>73</v>
@@ -2687,7 +2684,7 @@
         <v>74</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="J12" s="1">
         <v>1</v>
@@ -2696,7 +2693,7 @@
         <v>92</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="M12" s="1" t="s">
         <v>93</v>
@@ -2747,16 +2744,16 @@
         <v>92</v>
       </c>
       <c r="AF12" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AG12" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="AH12" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI12" s="5">
-        <v>6203</v>
+        <v>1</v>
+      </c>
+      <c r="AI12" s="5" t="s">
+        <v>142</v>
       </c>
       <c r="AJ12" s="1">
         <v>20</v>
@@ -2788,7 +2785,7 @@
         <v>45</v>
       </c>
       <c r="B13" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>73</v>
@@ -2803,7 +2800,7 @@
         <v>74</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="J13" s="1">
         <v>1</v>
@@ -2812,7 +2809,7 @@
         <v>92</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="M13" s="1" t="s">
         <v>93</v>
@@ -2863,16 +2860,16 @@
         <v>92</v>
       </c>
       <c r="AF13" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AG13" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="AH13" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI13" s="5">
-        <v>2341</v>
+        <v>1</v>
+      </c>
+      <c r="AI13" s="5" t="s">
+        <v>142</v>
       </c>
       <c r="AJ13" s="1">
         <v>20</v>
@@ -2880,8 +2877,8 @@
       <c r="AK13" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="AL13" s="5">
-        <v>6203</v>
+      <c r="AL13" s="5" t="s">
+        <v>86</v>
       </c>
       <c r="AM13" s="1">
         <v>8</v>

</xml_diff>

<commit_message>
Close #75: Take NrOfLdgs value instead hard-coded 1 landing for the quantity Added LandingTaxOnStartLocationRule and VsfFeeOnStartLocationRule to catch nr of landings on start location Added more unit tests for motor flight testing and implemented master data feeder for xlsx files
</commit_message>
<xml_diff>
--- a/flsserver/src/FLS.Server.Tests/TestData/FlightInvoiceTestdata_SGN.xlsx
+++ b/flsserver/src/FLS.Server.Tests/TestData/FlightInvoiceTestdata_SGN.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="146">
   <si>
     <t>UseCase</t>
   </si>
@@ -2024,10 +2024,10 @@
         <v>98</v>
       </c>
       <c r="P6" s="1">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="Q6" s="1" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="R6" s="1" t="s">
         <v>84</v>
@@ -2042,7 +2042,7 @@
         <v>300</v>
       </c>
       <c r="V6" s="1" t="s">
-        <v>103</v>
+        <v>72</v>
       </c>
       <c r="W6" s="1" t="s">
         <v>85</v>
@@ -2063,7 +2063,7 @@
         <v>1</v>
       </c>
       <c r="AD6" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AE6" s="1" t="s">
         <v>102</v>
@@ -2072,45 +2072,36 @@
         <v>124</v>
       </c>
       <c r="AG6" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="AH6" s="1">
         <v>0</v>
       </c>
-      <c r="AI6" s="5">
-        <v>2341</v>
+      <c r="AI6" s="5" t="s">
+        <v>104</v>
       </c>
       <c r="AJ6" s="1">
-        <v>180</v>
+        <v>5</v>
       </c>
       <c r="AK6" s="1" t="s">
         <v>67</v>
       </c>
       <c r="AL6" s="5" t="s">
-        <v>104</v>
+        <v>86</v>
       </c>
       <c r="AM6" s="1">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="AN6" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="AO6" s="5" t="s">
-        <v>86</v>
+      <c r="AO6" s="5">
+        <v>6203</v>
       </c>
       <c r="AP6" s="1">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AQ6" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AR6" s="5">
-        <v>6203</v>
-      </c>
-      <c r="AS6" s="1">
-        <v>1</v>
-      </c>
-      <c r="AT6" s="1" t="s">
         <v>68</v>
       </c>
     </row>
@@ -2583,10 +2574,10 @@
         <v>98</v>
       </c>
       <c r="P11" s="1">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="Q11" s="1" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="R11" s="1" t="s">
         <v>84</v>
@@ -2601,7 +2592,7 @@
         <v>180</v>
       </c>
       <c r="V11" s="1" t="s">
-        <v>103</v>
+        <v>72</v>
       </c>
       <c r="W11" s="1" t="s">
         <v>85</v>
@@ -2622,7 +2613,7 @@
         <v>1</v>
       </c>
       <c r="AD11" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AE11" s="1" t="s">
         <v>102</v>
@@ -2631,36 +2622,27 @@
         <v>124</v>
       </c>
       <c r="AG11" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="AH11" s="1">
         <v>0</v>
       </c>
-      <c r="AI11" s="5">
-        <v>2341</v>
+      <c r="AI11" s="5" t="s">
+        <v>104</v>
       </c>
       <c r="AJ11" s="1">
-        <v>180</v>
+        <v>3</v>
       </c>
       <c r="AK11" s="1" t="s">
         <v>67</v>
       </c>
       <c r="AL11" s="5" t="s">
-        <v>104</v>
+        <v>144</v>
       </c>
       <c r="AM11" s="1">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="AN11" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AO11" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="AP11" s="1">
-        <v>25</v>
-      </c>
-      <c r="AQ11" s="1" t="s">
         <v>67</v>
       </c>
     </row>

</xml_diff>